<commit_message>
added import to Eclipse slide
</commit_message>
<xml_diff>
--- a/Scottish MOD1_timings.xlsx
+++ b/Scottish MOD1_timings.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\Scotland\2025 Scotland Level 8 courses\Mod-1 Java Course New\Scottish Mod1 By Mike\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\2026 QA courses\Scotland\2025 Scotland Level 8 courses\Mod-1 Java Course New\Scottish Mod1 By Mike\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13DF178-9127-429E-B217-85BA671F5FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F721A8F1-BDAF-4C87-9C4E-01FC83A7A3ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -576,6 +576,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
@@ -585,7 +586,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -926,7 +926,7 @@
       <c r="F3" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="25" t="s">
         <v>47</v>
       </c>
     </row>
@@ -950,7 +950,7 @@
       <c r="F4" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="24"/>
+      <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
@@ -972,7 +972,7 @@
       <c r="F5" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="G5" s="24"/>
+      <c r="G5" s="25"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
@@ -992,7 +992,7 @@
         <v>6</v>
       </c>
       <c r="F6" s="19"/>
-      <c r="G6" s="24"/>
+      <c r="G6" s="25"/>
     </row>
     <row r="7" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
@@ -1014,7 +1014,7 @@
       <c r="F7" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="24"/>
+      <c r="G7" s="25"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
@@ -1033,7 +1033,7 @@
       <c r="E8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G8" s="24"/>
+      <c r="G8" s="25"/>
     </row>
     <row r="9" spans="1:7" s="15" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
@@ -1055,7 +1055,7 @@
       <c r="F9" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="G9" s="24"/>
+      <c r="G9" s="25"/>
     </row>
     <row r="10" spans="1:7" s="15" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
@@ -1075,7 +1075,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="20"/>
-      <c r="G10" s="24"/>
+      <c r="G10" s="25"/>
     </row>
     <row r="11" spans="1:7" s="15" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
@@ -1097,7 +1097,7 @@
       <c r="F11" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="G11" s="24"/>
+      <c r="G11" s="25"/>
     </row>
     <row r="12" spans="1:7" s="15" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
@@ -1119,7 +1119,7 @@
       <c r="F12" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="24"/>
+      <c r="G12" s="25"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
@@ -1138,7 +1138,7 @@
       <c r="E13" t="s">
         <v>58</v>
       </c>
-      <c r="G13" s="24"/>
+      <c r="G13" s="25"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
@@ -1155,13 +1155,13 @@
         <v>8</v>
       </c>
       <c r="F14" s="19"/>
-      <c r="G14" s="24"/>
+      <c r="G14" s="25"/>
     </row>
     <row r="15" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G15" s="24"/>
+      <c r="G15" s="25"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G16" s="24"/>
+      <c r="G16" s="25"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
@@ -1215,7 +1215,7 @@
       <c r="F20" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="24" t="s">
+      <c r="G20" s="25" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       <c r="F21" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="G21" s="24"/>
+      <c r="G21" s="25"/>
     </row>
     <row r="22" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
@@ -1255,7 +1255,7 @@
       <c r="D22" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G22" s="24"/>
+      <c r="G22" s="25"/>
     </row>
     <row r="23" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
@@ -1277,7 +1277,7 @@
       <c r="F23" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="G23" s="24"/>
+      <c r="G23" s="25"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
@@ -1296,7 +1296,7 @@
       <c r="E24" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G24" s="24"/>
+      <c r="G24" s="25"/>
     </row>
     <row r="25" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
@@ -1318,7 +1318,7 @@
       <c r="F25" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G25" s="24"/>
+      <c r="G25" s="25"/>
     </row>
     <row r="26" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5">
@@ -1340,7 +1340,7 @@
       <c r="F26" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="G26" s="24"/>
+      <c r="G26" s="25"/>
     </row>
     <row r="27" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
@@ -1359,7 +1359,7 @@
       <c r="E27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G27" s="24"/>
+      <c r="G27" s="25"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="5">
@@ -1381,7 +1381,7 @@
       <c r="F28" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G28" s="24"/>
+      <c r="G28" s="25"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="5">
@@ -1400,14 +1400,14 @@
       <c r="E29" t="s">
         <v>42</v>
       </c>
-      <c r="G29" s="24"/>
+      <c r="G29" s="25"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="5"/>
       <c r="B30" s="1"/>
       <c r="C30" s="5"/>
       <c r="D30" s="3"/>
-      <c r="G30" s="24"/>
+      <c r="G30" s="25"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="9"/>
@@ -1456,7 +1456,7 @@
       <c r="F33" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="G33" s="25" t="s">
+      <c r="G33" s="26" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       <c r="F34" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G34" s="25"/>
+      <c r="G34" s="26"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="5">
@@ -1500,7 +1500,7 @@
         <v>6</v>
       </c>
       <c r="F35" s="19"/>
-      <c r="G35" s="25"/>
+      <c r="G35" s="26"/>
     </row>
     <row r="36" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="5">
@@ -1522,7 +1522,7 @@
       <c r="F36" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="G36" s="25"/>
+      <c r="G36" s="26"/>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="5">
@@ -1544,7 +1544,7 @@
       <c r="F37" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="G37" s="25"/>
+      <c r="G37" s="26"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="5">
@@ -1563,7 +1563,7 @@
       <c r="E38" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G38" s="25"/>
+      <c r="G38" s="26"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="5">
@@ -1582,7 +1582,7 @@
       <c r="E39" t="s">
         <v>88</v>
       </c>
-      <c r="G39" s="25"/>
+      <c r="G39" s="26"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="5">
@@ -1604,7 +1604,7 @@
       <c r="F40" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G40" s="25"/>
+      <c r="G40" s="26"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="5">
@@ -1623,7 +1623,7 @@
       <c r="E41" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G41" s="25"/>
+      <c r="G41" s="26"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="5">
@@ -1645,7 +1645,7 @@
       <c r="F42" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G42" s="25"/>
+      <c r="G42" s="26"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="5">
@@ -1667,7 +1667,7 @@
       <c r="F43" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="G43" s="25"/>
+      <c r="G43" s="26"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="5">
@@ -1683,27 +1683,27 @@
       <c r="D44" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G44" s="25"/>
+      <c r="G44" s="26"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G45" s="25"/>
+      <c r="G45" s="26"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G46" s="25"/>
+      <c r="G46" s="26"/>
     </row>
     <row r="47" spans="1:7" s="15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B47" s="1">
         <f>B54+ TIME(0, C54, 0)</f>
         <v>0.46527777777777779</v>
       </c>
-      <c r="G47" s="25"/>
+      <c r="G47" s="26"/>
     </row>
     <row r="48" spans="1:7" s="15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="F48" s="20"/>
-      <c r="G48" s="25"/>
+      <c r="G48" s="26"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G49" s="25"/>
+      <c r="G49" s="26"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="10"/>
@@ -1752,7 +1752,7 @@
       <c r="F52" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="G52" s="25" t="s">
+      <c r="G52" s="26" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       <c r="F53" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="G53" s="25"/>
+      <c r="G53" s="26"/>
     </row>
     <row r="54" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54" s="5">
@@ -1798,7 +1798,7 @@
       <c r="F54" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="G54" s="25"/>
+      <c r="G54" s="26"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="5">
@@ -1817,7 +1817,7 @@
       <c r="E55" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G55" s="25"/>
+      <c r="G55" s="26"/>
     </row>
     <row r="56" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A56" s="5">
@@ -1839,7 +1839,7 @@
       <c r="F56" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="G56" s="25"/>
+      <c r="G56" s="26"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="5">
@@ -1859,7 +1859,7 @@
         <v>7</v>
       </c>
       <c r="F57" s="19"/>
-      <c r="G57" s="25"/>
+      <c r="G57" s="26"/>
     </row>
     <row r="58" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A58" s="5">
@@ -1881,7 +1881,7 @@
       <c r="F58" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="G58" s="25"/>
+      <c r="G58" s="26"/>
     </row>
     <row r="59" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A59" s="5">
@@ -1903,7 +1903,7 @@
       <c r="F59" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="G59" s="25"/>
+      <c r="G59" s="26"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="5">
@@ -1922,7 +1922,7 @@
       <c r="E60" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G60" s="25"/>
+      <c r="G60" s="26"/>
     </row>
     <row r="61" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A61" s="6">
@@ -1944,7 +1944,7 @@
       <c r="F61" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="G61" s="25"/>
+      <c r="G61" s="26"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="6"/>
@@ -1953,7 +1953,7 @@
         <v>0.67708333333333326</v>
       </c>
       <c r="C62" s="5"/>
-      <c r="G62" s="25"/>
+      <c r="G62" s="26"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="5">
@@ -1972,10 +1972,10 @@
       <c r="E63" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G63" s="25"/>
+      <c r="G63" s="26"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G64" s="25"/>
+      <c r="G64" s="26"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G65" s="22"/>
@@ -2027,7 +2027,7 @@
       <c r="F68" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="G68" s="26" t="s">
+      <c r="G68" s="27" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       <c r="F69" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="G69" s="26"/>
+      <c r="G69" s="27"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="5">
@@ -2070,7 +2070,7 @@
       <c r="E70" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G70" s="26"/>
+      <c r="G70" s="27"/>
     </row>
     <row r="71" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="5">
@@ -2092,7 +2092,7 @@
       <c r="F71" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="G71" s="26"/>
+      <c r="G71" s="27"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="5">
@@ -2111,7 +2111,7 @@
       <c r="E72" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G72" s="26"/>
+      <c r="G72" s="27"/>
     </row>
     <row r="73" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A73" s="5">
@@ -2133,7 +2133,7 @@
       <c r="F73" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="G73" s="26"/>
+      <c r="G73" s="27"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="5">
@@ -2152,7 +2152,7 @@
       <c r="E74" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G74" s="26"/>
+      <c r="G74" s="27"/>
     </row>
     <row r="75" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A75" s="5">
@@ -2174,7 +2174,7 @@
       <c r="F75" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G75" s="26"/>
+      <c r="G75" s="27"/>
     </row>
     <row r="76" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A76" s="5">
@@ -2196,7 +2196,7 @@
       <c r="F76" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G76" s="26"/>
+      <c r="G76" s="27"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="5">
@@ -2212,10 +2212,10 @@
       <c r="E77" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="G77" s="26"/>
+      <c r="G77" s="27"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G78" s="26"/>
+      <c r="G78" s="27"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="9"/>
@@ -2264,7 +2264,7 @@
       <c r="F81" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="G81" s="25" t="s">
+      <c r="G81" s="26" t="s">
         <v>52</v>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       <c r="F82" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="G82" s="25"/>
+      <c r="G82" s="26"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="5">
@@ -2307,7 +2307,7 @@
       <c r="E83" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G83" s="25"/>
+      <c r="G83" s="26"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="5">
@@ -2326,7 +2326,7 @@
       <c r="E84" t="s">
         <v>83</v>
       </c>
-      <c r="G84" s="25"/>
+      <c r="G84" s="26"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="5">
@@ -2345,7 +2345,7 @@
       <c r="E85" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G85" s="25"/>
+      <c r="G85" s="26"/>
     </row>
     <row r="86" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A86" s="5">
@@ -2367,7 +2367,7 @@
       <c r="F86" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="G86" s="25"/>
+      <c r="G86" s="26"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="5">
@@ -2386,7 +2386,7 @@
       <c r="E87" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G87" s="25"/>
+      <c r="G87" s="26"/>
     </row>
     <row r="88" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A88" s="5">
@@ -2408,7 +2408,7 @@
       <c r="F88" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="G88" s="25"/>
+      <c r="G88" s="26"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" s="5">
@@ -2427,7 +2427,7 @@
       <c r="E89" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G89" s="25"/>
+      <c r="G89" s="26"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="5"/>
@@ -2446,7 +2446,7 @@
       <c r="G91" s="12"/>
     </row>
     <row r="93" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="B93" s="27" t="s">
+      <c r="B93" s="24" t="s">
         <v>95</v>
       </c>
     </row>

</xml_diff>